<commit_message>
POS- Test Case 5 updated
</commit_message>
<xml_diff>
--- a/Test Results/Test_Result.xlsx
+++ b/Test Results/Test_Result.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>Method Name</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>28-12-2024</t>
+    <t>29-04-2025</t>
   </si>
   <si>
     <t>verifyHomeMenuVisibilityAfterLogin</t>
@@ -38,10 +38,7 @@
     <t>verifyCustomerNavigationAfterLogin</t>
   </si>
   <si>
-    <t>verifyCustomerDataEntry</t>
-  </si>
-  <si>
-    <t>Failed</t>
+    <t>testCaseFive</t>
   </si>
 </sst>
 </file>
@@ -58,7 +55,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,16 +72,6 @@
         <fgColor indexed="17"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -98,24 +85,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="33.71484375" customWidth="true" bestFit="true"/>
@@ -172,64 +154,9 @@
         <v>8</v>
       </c>
       <c r="B5" t="s" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s" s="5">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s" s="6">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s" s="7">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s" s="8">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>